<commit_message>
groupement d'activités et premier tests sur pondérations
</commit_message>
<xml_diff>
--- a/docs/downloads/04/tbl_age_obs_alaotra_ambatoharanana.xlsx
+++ b/docs/downloads/04/tbl_age_obs_alaotra_ambatoharanana.xlsx
@@ -495,12 +495,6 @@
           <t>61-70 ans</t>
         </is>
       </c>
-      <c r="C8">
-        <v>2</v>
-      </c>
-      <c r="D8">
-        <v>1.6</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -512,12 +506,6 @@
         <is>
           <t>71 ans et plus</t>
         </is>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9">
-        <v>0.8</v>
       </c>
     </row>
     <row r="10">

</xml_diff>